<commit_message>
Añadir opcion interactiva de colores especiales (+10%) para FLX-4155 y tejidos Flexol
</commit_message>
<xml_diff>
--- a/PRECIOS/FLEXOL ENERO 2026.xlsx
+++ b/PRECIOS/FLEXOL ENERO 2026.xlsx
@@ -452,7 +452,7 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -571,7 +571,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SCREENFLEX (Poliéster) - PL. 4155 (Colores especiales +10%)</t>
+          <t>SCREENFLEX (Poliéster) - PL. 4155</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -587,7 +587,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Mínimo a facturar 1,50 m² / Ud.</t>
+          <t>Colores especiales +10% | Mínimo 1,50 m²/Ud.</t>
         </is>
       </c>
     </row>

</xml_diff>